<commit_message>
final version. cleaned graphs, extra analysis
</commit_message>
<xml_diff>
--- a/Cost results_NEDdata1603.xlsx
+++ b/Cost results_NEDdata1603.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/laura_linuesa-domenech_tennet_eu/Documents/Thesis/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="706" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E74679F-8ABB-4403-8D0B-6A2826A939DB}"/>
+  <xr:revisionPtr revIDLastSave="708" documentId="8_{BA558C3F-E59C-4F04-9D2E-8441DAA40C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73392392-602B-4A7E-9CF4-5F6DEBD8145C}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{4AE1EDD8-8ACF-4AF9-86A6-B0088C54F040}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{4AE1EDD8-8ACF-4AF9-86A6-B0088C54F040}"/>
   </bookViews>
   <sheets>
     <sheet name="Rolling" sheetId="1" r:id="rId1"/>
@@ -309,7 +309,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -329,8 +329,6 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -690,7 +688,7 @@
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="18" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1408,7 +1406,7 @@
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="18" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2114,13 +2112,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B1" s="17" t="s">
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2170,8 +2168,8 @@
         <f>Fixed!C7</f>
         <v>81832480.922929183</v>
       </c>
-      <c r="D4" s="14">
-        <f t="shared" ref="D4:D5" si="0">(C4-B4)/B4</f>
+      <c r="D4" s="15">
+        <f t="shared" ref="D4" si="0">(C4-B4)/B4</f>
         <v>7.1951671764197841E-4</v>
       </c>
     </row>
@@ -2268,28 +2266,27 @@
         <v>0.16372959166745465</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="18"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>

</xml_diff>